<commit_message>
BEIJb.ST changed Excel file
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/BEIJb.ST.xlsx
+++ b/data/stx_xlsx/BEIJb.ST.xlsx
@@ -4209,7 +4209,7 @@
       <c r="Q36" s="18">
         <v>641.63</v>
       </c>
-      <c r="R36" s="17"/>
+      <c r="R36" s="18"/>
       <c r="S36" s="18">
         <v>443.56</v>
       </c>
@@ -4248,7 +4248,6 @@
       <c r="A37" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="B37" s="17"/>
       <c r="C37" s="18">
         <v>4569.37</v>
       </c>
@@ -4294,7 +4293,6 @@
       <c r="Q37" s="18">
         <v>641.63</v>
       </c>
-      <c r="R37" s="17"/>
       <c r="S37" s="18">
         <v>443.56</v>
       </c>
@@ -13982,7 +13980,9 @@
       <c r="A191" s="16" t="s">
         <v>250</v>
       </c>
-      <c r="B191" s="17"/>
+      <c r="B191" s="17">
+        <v>35453.35</v>
+      </c>
       <c r="C191" s="18">
         <v>4569.37</v>
       </c>
@@ -14028,7 +14028,9 @@
       <c r="Q191" s="18">
         <v>641.63</v>
       </c>
-      <c r="R191" s="17"/>
+      <c r="R191" s="18">
+        <v>3652.07</v>
+      </c>
       <c r="S191" s="18">
         <v>443.56</v>
       </c>

</xml_diff>